<commit_message>
Reroute to offshore_forecast_api and fix yearly forecast adjustment
</commit_message>
<xml_diff>
--- a/server/api/offshore_forecast_api/DATABASE PLATFORM.xlsx
+++ b/server/api/offshore_forecast_api/DATABASE PLATFORM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dzaki\Downloads\Forecast v3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dzaki\Downloads\offshore_forecast_api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06308066-46D2-49E4-8BC9-4A7A2343F14C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92CF25DC-47AE-438A-86B3-F896C7C374BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{A175ADA9-8FF9-49BC-836B-3AF0C9D9E775}"/>
   </bookViews>
@@ -282,8 +282,140 @@
 </comments>
 </file>
 
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Lugas Bijak Prasojo</author>
+    <author>Endang Widuri</author>
+  </authors>
+  <commentList>
+    <comment ref="J17" authorId="0" shapeId="0" xr:uid="{FA48AF56-191A-46DD-92DE-0BE9DABCCDE3}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Lugas Bijak Prasojo:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Included
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A22" authorId="0" shapeId="0" xr:uid="{2D19BB1B-AF7A-4EF6-93C7-56362C4E1D28}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Lugas Bijak Prasojo:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Braced Modular</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J23" authorId="0" shapeId="0" xr:uid="{01C42FB8-8C54-456B-8B4D-782BAB948094}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Lugas Bijak Prasojo:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Included in jacket</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I28" authorId="1" shapeId="0" xr:uid="{DD6164FB-9292-4D2D-A3CC-BF4947393B15}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Endang Widuri:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Deck Ext.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H29" authorId="1" shapeId="0" xr:uid="{63308B65-BFE2-4BA7-9B82-F9C62A00DC33}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Endang Widuri:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+incl Pile &amp; Cond</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="252">
   <si>
     <t>KKKS</t>
   </si>
@@ -1584,7 +1716,7 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1864,13 +1996,52 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1879,8 +2050,11 @@
     <xf numFmtId="0" fontId="17" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="199">
@@ -5321,121 +5495,121 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:110" ht="21" customHeight="1">
-      <c r="J1" s="96" t="s">
+      <c r="J1" s="113" t="s">
         <v>136</v>
       </c>
-      <c r="K1" s="96"/>
-      <c r="L1" s="96"/>
-      <c r="M1" s="97"/>
+      <c r="K1" s="113"/>
+      <c r="L1" s="113"/>
+      <c r="M1" s="114"/>
       <c r="N1" s="26"/>
-      <c r="O1" s="95" t="s">
+      <c r="O1" s="110" t="s">
         <v>137</v>
       </c>
-      <c r="P1" s="95"/>
-      <c r="Q1" s="95"/>
-      <c r="R1" s="95"/>
-      <c r="S1" s="95"/>
-      <c r="T1" s="95" t="s">
+      <c r="P1" s="110"/>
+      <c r="Q1" s="110"/>
+      <c r="R1" s="110"/>
+      <c r="S1" s="110"/>
+      <c r="T1" s="110" t="s">
         <v>138</v>
       </c>
-      <c r="U1" s="95"/>
-      <c r="V1" s="95"/>
-      <c r="W1" s="95"/>
-      <c r="X1" s="95"/>
-      <c r="Y1" s="95"/>
+      <c r="U1" s="110"/>
+      <c r="V1" s="110"/>
+      <c r="W1" s="110"/>
+      <c r="X1" s="110"/>
+      <c r="Y1" s="110"/>
       <c r="Z1" s="17"/>
-      <c r="AA1" s="95" t="s">
+      <c r="AA1" s="110" t="s">
         <v>139</v>
       </c>
-      <c r="AB1" s="95"/>
-      <c r="AC1" s="95"/>
-      <c r="AD1" s="95"/>
-      <c r="AE1" s="95"/>
-      <c r="AF1" s="95"/>
+      <c r="AB1" s="110"/>
+      <c r="AC1" s="110"/>
+      <c r="AD1" s="110"/>
+      <c r="AE1" s="110"/>
+      <c r="AF1" s="110"/>
       <c r="AG1" s="17"/>
-      <c r="AH1" s="95" t="s">
+      <c r="AH1" s="110" t="s">
         <v>140</v>
       </c>
-      <c r="AI1" s="95"/>
-      <c r="AJ1" s="95"/>
-      <c r="AK1" s="95"/>
-      <c r="AL1" s="95"/>
-      <c r="AM1" s="95"/>
-      <c r="AN1" s="95" t="s">
+      <c r="AI1" s="110"/>
+      <c r="AJ1" s="110"/>
+      <c r="AK1" s="110"/>
+      <c r="AL1" s="110"/>
+      <c r="AM1" s="110"/>
+      <c r="AN1" s="110" t="s">
         <v>141</v>
       </c>
-      <c r="AO1" s="95"/>
-      <c r="AP1" s="95"/>
-      <c r="AQ1" s="95"/>
-      <c r="AR1" s="95"/>
-      <c r="AS1" s="95"/>
-      <c r="AT1" s="95" t="s">
+      <c r="AO1" s="110"/>
+      <c r="AP1" s="110"/>
+      <c r="AQ1" s="110"/>
+      <c r="AR1" s="110"/>
+      <c r="AS1" s="110"/>
+      <c r="AT1" s="110" t="s">
         <v>142</v>
       </c>
-      <c r="AU1" s="95"/>
-      <c r="AV1" s="95"/>
-      <c r="AW1" s="95"/>
-      <c r="AX1" s="95"/>
-      <c r="AY1" s="95"/>
-      <c r="AZ1" s="95" t="s">
+      <c r="AU1" s="110"/>
+      <c r="AV1" s="110"/>
+      <c r="AW1" s="110"/>
+      <c r="AX1" s="110"/>
+      <c r="AY1" s="110"/>
+      <c r="AZ1" s="110" t="s">
         <v>143</v>
       </c>
-      <c r="BA1" s="95"/>
-      <c r="BB1" s="95"/>
-      <c r="BC1" s="95"/>
-      <c r="BD1" s="95"/>
-      <c r="BE1" s="95"/>
-      <c r="BF1" s="95" t="s">
+      <c r="BA1" s="110"/>
+      <c r="BB1" s="110"/>
+      <c r="BC1" s="110"/>
+      <c r="BD1" s="110"/>
+      <c r="BE1" s="110"/>
+      <c r="BF1" s="110" t="s">
         <v>144</v>
       </c>
-      <c r="BG1" s="95"/>
-      <c r="BH1" s="95"/>
-      <c r="BI1" s="95"/>
-      <c r="BJ1" s="95"/>
-      <c r="BK1" s="95"/>
-      <c r="BL1" s="95" t="s">
+      <c r="BG1" s="110"/>
+      <c r="BH1" s="110"/>
+      <c r="BI1" s="110"/>
+      <c r="BJ1" s="110"/>
+      <c r="BK1" s="110"/>
+      <c r="BL1" s="110" t="s">
         <v>145</v>
       </c>
-      <c r="BM1" s="95"/>
-      <c r="BN1" s="95"/>
-      <c r="BO1" s="95"/>
-      <c r="BP1" s="95"/>
-      <c r="BQ1" s="95"/>
+      <c r="BM1" s="110"/>
+      <c r="BN1" s="110"/>
+      <c r="BO1" s="110"/>
+      <c r="BP1" s="110"/>
+      <c r="BQ1" s="110"/>
       <c r="BR1" s="17"/>
-      <c r="BS1" s="95" t="s">
+      <c r="BS1" s="110" t="s">
         <v>146</v>
       </c>
-      <c r="BT1" s="95"/>
-      <c r="BU1" s="95"/>
-      <c r="BV1" s="95"/>
-      <c r="BW1" s="95"/>
-      <c r="BX1" s="95"/>
-      <c r="BY1" s="95"/>
+      <c r="BT1" s="110"/>
+      <c r="BU1" s="110"/>
+      <c r="BV1" s="110"/>
+      <c r="BW1" s="110"/>
+      <c r="BX1" s="110"/>
+      <c r="BY1" s="110"/>
       <c r="BZ1" s="17"/>
       <c r="CA1" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="CB1" s="95" t="s">
+      <c r="CB1" s="110" t="s">
         <v>148</v>
       </c>
-      <c r="CC1" s="95"/>
-      <c r="CD1" s="95"/>
-      <c r="CE1" s="95"/>
-      <c r="CF1" s="95"/>
-      <c r="CG1" s="95"/>
+      <c r="CC1" s="110"/>
+      <c r="CD1" s="110"/>
+      <c r="CE1" s="110"/>
+      <c r="CF1" s="110"/>
+      <c r="CG1" s="110"/>
       <c r="CH1" s="17"/>
       <c r="CI1" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="CJ1" s="95" t="s">
+      <c r="CJ1" s="110" t="s">
         <v>150</v>
       </c>
-      <c r="CK1" s="95"/>
-      <c r="CL1" s="95"/>
-      <c r="CM1" s="95"/>
-      <c r="CN1" s="95"/>
+      <c r="CK1" s="110"/>
+      <c r="CL1" s="110"/>
+      <c r="CM1" s="110"/>
+      <c r="CN1" s="110"/>
       <c r="CO1" s="28"/>
-      <c r="CP1" s="98" t="s">
+      <c r="CP1" s="111" t="s">
         <v>13</v>
       </c>
       <c r="CQ1" s="29"/>
@@ -5713,7 +5887,7 @@
       <c r="CO2" s="37" t="s">
         <v>251</v>
       </c>
-      <c r="CP2" s="99"/>
+      <c r="CP2" s="112"/>
       <c r="CQ2" s="38" t="s">
         <v>77</v>
       </c>
@@ -6125,7 +6299,7 @@
         <v>1795434.92</v>
       </c>
       <c r="CO4" s="43">
-        <f>SUM(CJ4:CN4)</f>
+        <f t="shared" ref="CO4:CO30" si="2">SUM(CJ4:CN4)</f>
         <v>56319587.670000002</v>
       </c>
       <c r="CP4" s="85">
@@ -6363,7 +6537,7 @@
         <v>291809113</v>
       </c>
       <c r="BY5" s="68">
-        <f t="shared" ref="BY5:BY25" si="2">SUM(BS5:BX5)</f>
+        <f t="shared" ref="BY5:BY25" si="3">SUM(BS5:BX5)</f>
         <v>824573232</v>
       </c>
       <c r="BZ5" s="44">
@@ -6411,7 +6585,7 @@
         <v>940849</v>
       </c>
       <c r="CO5" s="43">
-        <f>SUM(CJ5:CN5)</f>
+        <f t="shared" si="2"/>
         <v>142850662</v>
       </c>
       <c r="CP5" s="85">
@@ -6636,7 +6810,7 @@
         <v>138347198</v>
       </c>
       <c r="BY6" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>228902395</v>
       </c>
       <c r="BZ6" s="44">
@@ -6682,8 +6856,8 @@
       <c r="CN6" s="46">
         <v>139398</v>
       </c>
-      <c r="CO6" s="100">
-        <f>SUM(CJ6:CN6)</f>
+      <c r="CO6" s="95">
+        <f t="shared" si="2"/>
         <v>21980738</v>
       </c>
       <c r="CP6" s="85">
@@ -6910,7 +7084,7 @@
         <v>906887.59</v>
       </c>
       <c r="BY7" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1853658.31</v>
       </c>
       <c r="BZ7" s="44">
@@ -6958,7 +7132,7 @@
         <v>0</v>
       </c>
       <c r="CO7" s="43">
-        <f>SUM(CJ7:CN7)</f>
+        <f t="shared" si="2"/>
         <v>701734.02</v>
       </c>
       <c r="CP7" s="85">
@@ -7189,7 +7363,7 @@
         <v>26024403</v>
       </c>
       <c r="BY8" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>31818765</v>
       </c>
       <c r="BZ8" s="44">
@@ -7237,7 +7411,7 @@
         <v>0</v>
       </c>
       <c r="CO8" s="43">
-        <f>SUM(CJ8:CN8)</f>
+        <f t="shared" si="2"/>
         <v>14389464.77</v>
       </c>
       <c r="CP8" s="85">
@@ -7447,28 +7621,13 @@
         <v>0</v>
       </c>
       <c r="BR9" s="43"/>
-      <c r="BS9" s="42">
-        <v>0</v>
-      </c>
-      <c r="BT9" s="42">
-        <v>0</v>
-      </c>
-      <c r="BU9" s="42">
-        <v>0</v>
-      </c>
-      <c r="BV9" s="42">
-        <v>0</v>
-      </c>
-      <c r="BW9" s="42">
-        <v>0</v>
-      </c>
-      <c r="BX9" s="42">
-        <v>0</v>
-      </c>
-      <c r="BY9" s="68">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="BS9" s="42"/>
+      <c r="BT9" s="42"/>
+      <c r="BU9" s="42"/>
+      <c r="BV9" s="42"/>
+      <c r="BW9" s="42"/>
+      <c r="BX9" s="42"/>
+      <c r="BY9" s="68"/>
       <c r="BZ9" s="44"/>
       <c r="CA9" s="42">
         <v>0</v>
@@ -7511,7 +7670,7 @@
         <v>293109.49</v>
       </c>
       <c r="CO9" s="43">
-        <f>SUM(CJ9:CN9)</f>
+        <f t="shared" si="2"/>
         <v>2044031.64</v>
       </c>
       <c r="CP9" s="85">
@@ -7719,28 +7878,13 @@
         <v>0</v>
       </c>
       <c r="BR10" s="43"/>
-      <c r="BS10" s="42">
-        <v>0</v>
-      </c>
-      <c r="BT10" s="42">
-        <v>0</v>
-      </c>
-      <c r="BU10" s="42">
-        <v>0</v>
-      </c>
-      <c r="BV10" s="42">
-        <v>0</v>
-      </c>
-      <c r="BW10" s="42">
-        <v>0</v>
-      </c>
-      <c r="BX10" s="42">
-        <v>0</v>
-      </c>
-      <c r="BY10" s="68">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="BS10" s="42"/>
+      <c r="BT10" s="42"/>
+      <c r="BU10" s="42"/>
+      <c r="BV10" s="42"/>
+      <c r="BW10" s="42"/>
+      <c r="BX10" s="42"/>
+      <c r="BY10" s="68"/>
       <c r="BZ10" s="44"/>
       <c r="CA10" s="42">
         <v>0</v>
@@ -7783,7 +7927,7 @@
         <v>0</v>
       </c>
       <c r="CO10" s="43">
-        <f>SUM(CJ10:CN10)</f>
+        <f t="shared" si="2"/>
         <v>5179667</v>
       </c>
       <c r="CP10" s="85">
@@ -7989,28 +8133,13 @@
         <v>0</v>
       </c>
       <c r="BR11" s="43"/>
-      <c r="BS11" s="42">
-        <v>0</v>
-      </c>
-      <c r="BT11" s="42">
-        <v>0</v>
-      </c>
-      <c r="BU11" s="42">
-        <v>0</v>
-      </c>
-      <c r="BV11" s="42">
-        <v>0</v>
-      </c>
-      <c r="BW11" s="42">
-        <v>0</v>
-      </c>
-      <c r="BX11" s="42">
-        <v>0</v>
-      </c>
-      <c r="BY11" s="68">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="BS11" s="42"/>
+      <c r="BT11" s="42"/>
+      <c r="BU11" s="42"/>
+      <c r="BV11" s="42"/>
+      <c r="BW11" s="42"/>
+      <c r="BX11" s="42"/>
+      <c r="BY11" s="68"/>
       <c r="BZ11" s="44"/>
       <c r="CA11" s="42">
         <v>47643</v>
@@ -8053,7 +8182,7 @@
         <v>0</v>
       </c>
       <c r="CO11" s="43">
-        <f>SUM(CJ11:CN11)</f>
+        <f t="shared" si="2"/>
         <v>890782</v>
       </c>
       <c r="CP11" s="85">
@@ -8285,7 +8414,7 @@
         <v>8239301</v>
       </c>
       <c r="BY12" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>16068171</v>
       </c>
       <c r="BZ12" s="44">
@@ -8333,7 +8462,7 @@
         <v>0</v>
       </c>
       <c r="CO12" s="43">
-        <f>SUM(CJ12:CN12)</f>
+        <f t="shared" si="2"/>
         <v>3650031</v>
       </c>
       <c r="CP12" s="85">
@@ -8565,7 +8694,7 @@
         <v>7910234.2000000002</v>
       </c>
       <c r="BY13" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>15873860.940000001</v>
       </c>
       <c r="BZ13" s="44">
@@ -8613,7 +8742,7 @@
         <v>0</v>
       </c>
       <c r="CO13" s="43">
-        <f>SUM(CJ13:CN13)</f>
+        <f t="shared" si="2"/>
         <v>3744980</v>
       </c>
       <c r="CP13" s="85">
@@ -8845,11 +8974,11 @@
         <v>4929059</v>
       </c>
       <c r="BY14" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9512031.5600000005</v>
       </c>
       <c r="BZ14" s="44">
-        <f t="shared" ref="BZ14:BZ25" si="3">BY14/L14/N14</f>
+        <f t="shared" ref="BZ14:BZ25" si="4">BY14/L14/N14</f>
         <v>221210.03627906978</v>
       </c>
       <c r="CA14" s="42">
@@ -8893,7 +9022,7 @@
         <v>0</v>
       </c>
       <c r="CO14" s="43">
-        <f>SUM(CJ14:CN14)</f>
+        <f t="shared" si="2"/>
         <v>3847452.94</v>
       </c>
       <c r="CP14" s="85">
@@ -9131,11 +9260,11 @@
         <v>12002302</v>
       </c>
       <c r="BY15" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>18456623</v>
       </c>
       <c r="BZ15" s="44">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>384512.97916666669</v>
       </c>
       <c r="CA15" s="42">
@@ -9179,7 +9308,7 @@
         <v>0</v>
       </c>
       <c r="CO15" s="43">
-        <f>SUM(CJ15:CN15)</f>
+        <f t="shared" si="2"/>
         <v>4819880</v>
       </c>
       <c r="CP15" s="85">
@@ -9417,11 +9546,11 @@
         <v>12297645</v>
       </c>
       <c r="BY16" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>19282247</v>
       </c>
       <c r="BZ16" s="44">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>297565.5401234568</v>
       </c>
       <c r="CA16" s="42">
@@ -9465,7 +9594,7 @@
         <v>0</v>
       </c>
       <c r="CO16" s="43">
-        <f>SUM(CJ16:CN16)</f>
+        <f t="shared" si="2"/>
         <v>4760885</v>
       </c>
       <c r="CP16" s="85">
@@ -9703,11 +9832,11 @@
         <v>12434012</v>
       </c>
       <c r="BY17" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>19407341</v>
       </c>
       <c r="BZ17" s="44">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>299496.00308641978</v>
       </c>
       <c r="CA17" s="42">
@@ -9751,7 +9880,7 @@
         <v>0</v>
       </c>
       <c r="CO17" s="43">
-        <f>SUM(CJ17:CN17)</f>
+        <f t="shared" si="2"/>
         <v>4462892</v>
       </c>
       <c r="CP17" s="85">
@@ -9982,11 +10111,11 @@
         <v>12658516.640000001</v>
       </c>
       <c r="BY18" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>20629655</v>
       </c>
       <c r="BZ18" s="44">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>491182.26190476195</v>
       </c>
       <c r="CA18" s="42">
@@ -10030,7 +10159,7 @@
         <v>0</v>
       </c>
       <c r="CO18" s="43">
-        <f>SUM(CJ18:CN18)</f>
+        <f t="shared" si="2"/>
         <v>8882950.6699999999</v>
       </c>
       <c r="CP18" s="85">
@@ -10259,11 +10388,11 @@
         <v>6346024.6100000003</v>
       </c>
       <c r="BY19" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>10656112.940000001</v>
       </c>
       <c r="BZ19" s="44">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1776018.8233333335</v>
       </c>
       <c r="CA19" s="42">
@@ -10307,7 +10436,7 @@
         <v>0</v>
       </c>
       <c r="CO19" s="43">
-        <f>SUM(CJ19:CN19)</f>
+        <f t="shared" si="2"/>
         <v>29138732</v>
       </c>
       <c r="CP19" s="85">
@@ -10541,7 +10670,7 @@
         <v>6141245.04</v>
       </c>
       <c r="BY20" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6558041.1399999997</v>
       </c>
       <c r="BZ20" s="44">
@@ -10589,7 +10718,7 @@
         <v>973522.08</v>
       </c>
       <c r="CO20" s="43">
-        <f>SUM(CJ20:CN20)</f>
+        <f t="shared" si="2"/>
         <v>2515345.5699999998</v>
       </c>
       <c r="CP20" s="85">
@@ -10820,11 +10949,11 @@
         <v>15992522</v>
       </c>
       <c r="BY21" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>25641953</v>
       </c>
       <c r="BZ21" s="44">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>77351.291101055802</v>
       </c>
       <c r="CA21" s="42">
@@ -10868,7 +10997,7 @@
         <v>447344</v>
       </c>
       <c r="CO21" s="43">
-        <f>SUM(CJ21:CN21)</f>
+        <f t="shared" si="2"/>
         <v>4708129</v>
       </c>
       <c r="CP21" s="85">
@@ -11103,11 +11232,11 @@
         <v>9314224.4000000004</v>
       </c>
       <c r="BY22" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>15008912.32</v>
       </c>
       <c r="BZ22" s="44">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>110359.64941176471</v>
       </c>
       <c r="CA22" s="42">
@@ -11151,7 +11280,7 @@
         <v>3845675.91</v>
       </c>
       <c r="CO22" s="43">
-        <f>SUM(CJ22:CN22)</f>
+        <f t="shared" si="2"/>
         <v>13004148.340000002</v>
       </c>
       <c r="CP22" s="85">
@@ -11381,11 +11510,11 @@
         <v>15442067.470000001</v>
       </c>
       <c r="BY23" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>18641195.150000002</v>
       </c>
       <c r="BZ23" s="44">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>408798.13925438607</v>
       </c>
       <c r="CA23" s="42">
@@ -11429,7 +11558,7 @@
         <v>0</v>
       </c>
       <c r="CO23" s="43">
-        <f>SUM(CJ23:CN23)</f>
+        <f t="shared" si="2"/>
         <v>6314776.7400000002</v>
       </c>
       <c r="CP23" s="85">
@@ -11660,11 +11789,11 @@
         <v>16099331.289999999</v>
       </c>
       <c r="BY24" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>24787400.779999997</v>
       </c>
       <c r="BZ24" s="44">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>167936.31964769645</v>
       </c>
       <c r="CA24" s="42">
@@ -11708,7 +11837,7 @@
         <v>1559912.48</v>
       </c>
       <c r="CO24" s="43">
-        <f>SUM(CJ24:CN24)</f>
+        <f t="shared" si="2"/>
         <v>9171013.3599999994</v>
       </c>
       <c r="CP24" s="85">
@@ -11942,11 +12071,11 @@
         <v>29085237.5</v>
       </c>
       <c r="BY25" s="68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>70165662.669999987</v>
       </c>
       <c r="BZ25" s="44">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>92811.72310846558</v>
       </c>
       <c r="CA25" s="42">
@@ -11990,7 +12119,7 @@
         <v>2246699.7200000002</v>
       </c>
       <c r="CO25" s="43">
-        <f>SUM(CJ25:CN25)</f>
+        <f t="shared" si="2"/>
         <v>14929309.390000001</v>
       </c>
       <c r="CP25" s="85">
@@ -12254,8 +12383,8 @@
       <c r="CN26" s="46">
         <v>822591</v>
       </c>
-      <c r="CO26" s="100">
-        <f>SUM(CJ26:CN26)</f>
+      <c r="CO26" s="95">
+        <f t="shared" si="2"/>
         <v>9839512</v>
       </c>
       <c r="CP26" s="86">
@@ -12520,8 +12649,8 @@
       <c r="CN27" s="46">
         <v>822591</v>
       </c>
-      <c r="CO27" s="100">
-        <f>SUM(CJ27:CN27)</f>
+      <c r="CO27" s="95">
+        <f t="shared" si="2"/>
         <v>9859101</v>
       </c>
       <c r="CP27" s="85">
@@ -12750,7 +12879,7 @@
         <v>13075370.307612393</v>
       </c>
       <c r="BY28" s="69">
-        <f t="shared" ref="BY28" si="4">SUM(BS28:BX28)</f>
+        <f t="shared" ref="BY28" si="5">SUM(BS28:BX28)</f>
         <v>22871416.555628229</v>
       </c>
       <c r="BZ28" s="44">
@@ -12797,7 +12926,7 @@
         <v>118925.36</v>
       </c>
       <c r="CO28" s="61">
-        <f>SUM(CJ28:CN28)</f>
+        <f t="shared" si="2"/>
         <v>8150562.5900000008</v>
       </c>
       <c r="CP28" s="87">
@@ -12894,7 +13023,7 @@
         <v>0</v>
       </c>
       <c r="AG29" s="47">
-        <f t="shared" ref="AG29:AG30" si="5">SUM(AB29:AF29)</f>
+        <f t="shared" ref="AG29:AG30" si="6">SUM(AB29:AF29)</f>
         <v>0</v>
       </c>
       <c r="AH29" s="46">
@@ -12970,7 +13099,7 @@
         <v>0</v>
       </c>
       <c r="BE29" s="47">
-        <f t="shared" ref="BE29:BE30" si="6">SUM(AZ29:BD29)</f>
+        <f t="shared" ref="BE29:BE30" si="7">SUM(AZ29:BD29)</f>
         <v>0</v>
       </c>
       <c r="BF29" s="46">
@@ -12989,7 +13118,7 @@
         <v>0</v>
       </c>
       <c r="BK29" s="71">
-        <f t="shared" ref="BK29:BK30" si="7">SUM(BF29:BJ29)</f>
+        <f t="shared" ref="BK29:BK30" si="8">SUM(BF29:BJ29)</f>
         <v>0</v>
       </c>
       <c r="BL29" s="46">
@@ -13062,7 +13191,7 @@
         <v>0</v>
       </c>
       <c r="CH29" s="61">
-        <f t="shared" ref="CH29:CH30" si="8">SUM(CC29:CG29)</f>
+        <f t="shared" ref="CH29:CH30" si="9">SUM(CC29:CG29)</f>
         <v>0</v>
       </c>
       <c r="CI29" s="62">
@@ -13084,7 +13213,7 @@
         <v>0</v>
       </c>
       <c r="CO29" s="61">
-        <f>SUM(CJ29:CN29)</f>
+        <f t="shared" si="2"/>
         <v>12566347</v>
       </c>
       <c r="CP29" s="87">
@@ -13171,7 +13300,7 @@
         <v>0</v>
       </c>
       <c r="AG30" s="47">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AH30" s="46">
@@ -13247,7 +13376,7 @@
         <v>0</v>
       </c>
       <c r="BE30" s="47">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="BF30" s="46">
@@ -13266,7 +13395,7 @@
         <v>0</v>
       </c>
       <c r="BK30" s="71">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="BL30" s="46">
@@ -13336,7 +13465,7 @@
         <v>0</v>
       </c>
       <c r="CH30" s="61">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="CI30" s="62">
@@ -13358,7 +13487,7 @@
         <v>0</v>
       </c>
       <c r="CO30" s="61">
-        <f>SUM(CJ30:CN30)</f>
+        <f t="shared" si="2"/>
         <v>35162073.956102334</v>
       </c>
       <c r="CP30" s="87">
@@ -13777,6 +13906,12 @@
   </sheetData>
   <autoFilter ref="A2:DF2" xr:uid="{FE5FCFA7-2727-46F1-BA8C-34C3979F0D07}"/>
   <mergeCells count="14">
+    <mergeCell ref="AN1:AS1"/>
+    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="O1:S1"/>
+    <mergeCell ref="T1:Y1"/>
+    <mergeCell ref="AA1:AF1"/>
+    <mergeCell ref="AH1:AM1"/>
     <mergeCell ref="CJ1:CN1"/>
     <mergeCell ref="CP1:CP2"/>
     <mergeCell ref="AT1:AY1"/>
@@ -13785,12 +13920,6 @@
     <mergeCell ref="BL1:BQ1"/>
     <mergeCell ref="BS1:BY1"/>
     <mergeCell ref="CB1:CG1"/>
-    <mergeCell ref="AN1:AS1"/>
-    <mergeCell ref="J1:M1"/>
-    <mergeCell ref="O1:S1"/>
-    <mergeCell ref="T1:Y1"/>
-    <mergeCell ref="AA1:AF1"/>
-    <mergeCell ref="AH1:AM1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="CQ20" r:id="rId1" display="https://newafe.skkmigas.go.id/home/document-viewer/inline/3af14e24-b803-40be-8537-ab336785717f" xr:uid="{A4553338-6786-8946-9112-0E028144465A}"/>
@@ -13827,65 +13956,1028 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99FC28B5-5343-4149-8359-4C5C5F905BC5}">
-  <dimension ref="A1:T1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99FC28B5-5343-4149-8359-4C5C5F905BC5}">
+  <dimension ref="A1:S29"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="15" thickBot="1">
-      <c r="A1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="1">
-        <v>4</v>
-      </c>
-      <c r="F1" s="5">
-        <v>60</v>
-      </c>
-      <c r="G1" s="89" t="s">
-        <v>177</v>
-      </c>
-      <c r="H1" s="89">
-        <v>24</v>
-      </c>
-      <c r="I1" s="3">
-        <v>2270</v>
-      </c>
-      <c r="J1" s="3">
-        <v>3881</v>
-      </c>
-      <c r="K1" s="3">
-        <v>3238</v>
-      </c>
-      <c r="L1" s="75">
-        <v>0</v>
+    <row r="1" spans="1:19" ht="43.5">
+      <c r="A1" s="96" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="84" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="97" t="s">
+        <v>154</v>
+      </c>
+      <c r="D1" s="97"/>
+      <c r="E1" s="97" t="s">
+        <v>155</v>
+      </c>
+      <c r="F1" s="97"/>
+      <c r="G1" s="98" t="s">
+        <v>156</v>
+      </c>
+      <c r="H1" s="98" t="s">
+        <v>157</v>
+      </c>
+      <c r="I1" s="98" t="s">
+        <v>158</v>
+      </c>
+      <c r="J1" s="97" t="s">
+        <v>159</v>
+      </c>
+      <c r="K1" s="97" t="s">
+        <v>160</v>
       </c>
       <c r="M1" s="75"/>
       <c r="N1" s="75"/>
       <c r="O1" s="75"/>
       <c r="P1" s="75"/>
-      <c r="Q1" s="75">
-        <f t="shared" ref="Q1" si="0">R1-(SUM(L1:P1))</f>
-        <v>0</v>
-      </c>
-      <c r="R1" s="23"/>
-      <c r="S1" s="16" t="s">
-        <v>78</v>
-      </c>
-      <c r="T1" s="3"/>
+      <c r="Q1" s="23"/>
+      <c r="R1" s="16"/>
+      <c r="S1" s="3"/>
+    </row>
+    <row r="2" spans="1:19" ht="43.5">
+      <c r="A2" s="99">
+        <v>4</v>
+      </c>
+      <c r="B2" s="100">
+        <v>60</v>
+      </c>
+      <c r="C2" s="101" t="s">
+        <v>177</v>
+      </c>
+      <c r="D2" s="101"/>
+      <c r="E2" s="101" t="s">
+        <v>178</v>
+      </c>
+      <c r="F2" s="101">
+        <v>24</v>
+      </c>
+      <c r="G2" s="102">
+        <v>2270</v>
+      </c>
+      <c r="H2" s="102">
+        <v>3881</v>
+      </c>
+      <c r="I2" s="102">
+        <v>3238</v>
+      </c>
+      <c r="J2" s="12">
+        <v>1386</v>
+      </c>
+      <c r="K2" s="12">
+        <f t="shared" ref="K2:K27" si="0">SUM(G2:J2)</f>
+        <v>10775</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19">
+      <c r="A3" s="103">
+        <v>6</v>
+      </c>
+      <c r="B3" s="100">
+        <v>57</v>
+      </c>
+      <c r="C3" s="101" t="s">
+        <v>181</v>
+      </c>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101" t="s">
+        <v>178</v>
+      </c>
+      <c r="F3" s="101">
+        <v>24</v>
+      </c>
+      <c r="G3" s="102">
+        <v>4052</v>
+      </c>
+      <c r="H3" s="102">
+        <v>3450</v>
+      </c>
+      <c r="I3" s="102">
+        <v>3665</v>
+      </c>
+      <c r="J3" s="12">
+        <v>2480</v>
+      </c>
+      <c r="K3" s="12">
+        <f t="shared" si="0"/>
+        <v>13647</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" ht="43.5">
+      <c r="A4" s="99">
+        <v>4</v>
+      </c>
+      <c r="B4" s="100">
+        <v>40</v>
+      </c>
+      <c r="C4" s="101" t="s">
+        <v>184</v>
+      </c>
+      <c r="D4" s="101">
+        <f>67.2+3.5+12.1</f>
+        <v>82.8</v>
+      </c>
+      <c r="E4" s="101" t="s">
+        <v>185</v>
+      </c>
+      <c r="F4" s="101">
+        <v>24</v>
+      </c>
+      <c r="G4" s="102">
+        <f>2377+1715</f>
+        <v>4092</v>
+      </c>
+      <c r="H4" s="102">
+        <f>1172+1062</f>
+        <v>2234</v>
+      </c>
+      <c r="I4" s="102">
+        <f>1148+1123</f>
+        <v>2271</v>
+      </c>
+      <c r="J4" s="12">
+        <f>326+255</f>
+        <v>581</v>
+      </c>
+      <c r="K4" s="12">
+        <f t="shared" si="0"/>
+        <v>9178</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19">
+      <c r="A5" s="99">
+        <v>4</v>
+      </c>
+      <c r="B5" s="100">
+        <v>40</v>
+      </c>
+      <c r="C5" s="101" t="s">
+        <v>247</v>
+      </c>
+      <c r="D5" s="101"/>
+      <c r="E5" s="101" t="s">
+        <v>226</v>
+      </c>
+      <c r="F5" s="101"/>
+      <c r="G5" s="102">
+        <v>1836</v>
+      </c>
+      <c r="H5" s="102">
+        <v>1699</v>
+      </c>
+      <c r="I5" s="102">
+        <v>1588</v>
+      </c>
+      <c r="J5" s="12">
+        <v>378</v>
+      </c>
+      <c r="K5" s="12">
+        <f t="shared" si="0"/>
+        <v>5501</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19">
+      <c r="A6" s="99">
+        <v>4</v>
+      </c>
+      <c r="B6" s="100">
+        <v>4</v>
+      </c>
+      <c r="C6" s="104" t="s">
+        <v>187</v>
+      </c>
+      <c r="D6" s="104"/>
+      <c r="E6" s="104" t="s">
+        <v>188</v>
+      </c>
+      <c r="F6" s="104">
+        <v>6</v>
+      </c>
+      <c r="G6" s="102">
+        <v>160.13</v>
+      </c>
+      <c r="H6" s="102">
+        <v>0</v>
+      </c>
+      <c r="I6" s="102">
+        <v>110</v>
+      </c>
+      <c r="J6" s="12">
+        <v>0</v>
+      </c>
+      <c r="K6" s="12">
+        <f t="shared" si="0"/>
+        <v>270.13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19">
+      <c r="A7" s="99">
+        <v>4</v>
+      </c>
+      <c r="B7" s="100">
+        <v>57.2</v>
+      </c>
+      <c r="C7" s="104" t="s">
+        <v>191</v>
+      </c>
+      <c r="D7" s="104"/>
+      <c r="E7" s="104" t="s">
+        <v>192</v>
+      </c>
+      <c r="F7" s="104">
+        <v>16</v>
+      </c>
+      <c r="G7" s="102">
+        <v>2100</v>
+      </c>
+      <c r="H7" s="102">
+        <v>1536</v>
+      </c>
+      <c r="I7" s="102">
+        <v>1685</v>
+      </c>
+      <c r="J7" s="12">
+        <v>0</v>
+      </c>
+      <c r="K7" s="12">
+        <f t="shared" si="0"/>
+        <v>5321</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19">
+      <c r="A8" s="99">
+        <v>3</v>
+      </c>
+      <c r="B8" s="100">
+        <v>76</v>
+      </c>
+      <c r="C8" s="104" t="s">
+        <v>194</v>
+      </c>
+      <c r="D8" s="104"/>
+      <c r="E8" s="104">
+        <v>10</v>
+      </c>
+      <c r="F8" s="104">
+        <v>10</v>
+      </c>
+      <c r="G8" s="102">
+        <v>97.6</v>
+      </c>
+      <c r="H8" s="102">
+        <v>800.44500000000005</v>
+      </c>
+      <c r="I8" s="102">
+        <v>0</v>
+      </c>
+      <c r="J8" s="12">
+        <v>0</v>
+      </c>
+      <c r="K8" s="12">
+        <f t="shared" si="0"/>
+        <v>898.04500000000007</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19">
+      <c r="A9" s="99">
+        <v>4</v>
+      </c>
+      <c r="B9" s="100">
+        <v>103</v>
+      </c>
+      <c r="C9" s="104" t="s">
+        <v>181</v>
+      </c>
+      <c r="D9" s="104"/>
+      <c r="E9" s="104" t="s">
+        <v>195</v>
+      </c>
+      <c r="F9" s="104">
+        <v>20</v>
+      </c>
+      <c r="G9" s="102">
+        <v>222</v>
+      </c>
+      <c r="H9" s="102">
+        <v>2188</v>
+      </c>
+      <c r="I9" s="102">
+        <v>0</v>
+      </c>
+      <c r="J9" s="12">
+        <v>0</v>
+      </c>
+      <c r="K9" s="12">
+        <f t="shared" si="0"/>
+        <v>2410</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19">
+      <c r="A10" s="99">
+        <v>3</v>
+      </c>
+      <c r="B10" s="100">
+        <v>70</v>
+      </c>
+      <c r="C10" s="104" t="s">
+        <v>246</v>
+      </c>
+      <c r="D10" s="104"/>
+      <c r="E10" s="104" t="s">
+        <v>199</v>
+      </c>
+      <c r="F10" s="104"/>
+      <c r="G10" s="102">
+        <v>75</v>
+      </c>
+      <c r="H10" s="102">
+        <v>600</v>
+      </c>
+      <c r="I10" s="102">
+        <v>550</v>
+      </c>
+      <c r="J10" s="12">
+        <v>0</v>
+      </c>
+      <c r="K10" s="12">
+        <f t="shared" si="0"/>
+        <v>1225</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19">
+      <c r="A11" s="99">
+        <v>3</v>
+      </c>
+      <c r="B11" s="100">
+        <v>50.8</v>
+      </c>
+      <c r="C11" s="104" t="s">
+        <v>198</v>
+      </c>
+      <c r="D11" s="104">
+        <v>6.79</v>
+      </c>
+      <c r="E11" s="104" t="s">
+        <v>199</v>
+      </c>
+      <c r="F11" s="104">
+        <v>10</v>
+      </c>
+      <c r="G11" s="102">
+        <v>276.93</v>
+      </c>
+      <c r="H11" s="102">
+        <f>613.7+118.49</f>
+        <v>732.19</v>
+      </c>
+      <c r="I11" s="102">
+        <v>570.35</v>
+      </c>
+      <c r="J11" s="12">
+        <v>316.7</v>
+      </c>
+      <c r="K11" s="12">
+        <f t="shared" si="0"/>
+        <v>1896.1700000000003</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19">
+      <c r="A12" s="99">
+        <v>3</v>
+      </c>
+      <c r="B12" s="100">
+        <v>62.9</v>
+      </c>
+      <c r="C12" s="104" t="s">
+        <v>201</v>
+      </c>
+      <c r="D12" s="104">
+        <v>5</v>
+      </c>
+      <c r="E12" s="104" t="s">
+        <v>199</v>
+      </c>
+      <c r="F12" s="104">
+        <v>10</v>
+      </c>
+      <c r="G12" s="102">
+        <v>334.78800000000001</v>
+      </c>
+      <c r="H12" s="102">
+        <f>716.74+94.58</f>
+        <v>811.32</v>
+      </c>
+      <c r="I12" s="102">
+        <v>598.69000000000005</v>
+      </c>
+      <c r="J12" s="12">
+        <v>362.31</v>
+      </c>
+      <c r="K12" s="12">
+        <f t="shared" si="0"/>
+        <v>2107.1080000000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19">
+      <c r="A13" s="99">
+        <v>3</v>
+      </c>
+      <c r="B13" s="100">
+        <v>71.7</v>
+      </c>
+      <c r="C13" s="104" t="s">
+        <v>203</v>
+      </c>
+      <c r="D13" s="104">
+        <v>4.3</v>
+      </c>
+      <c r="E13" s="104" t="s">
+        <v>199</v>
+      </c>
+      <c r="F13" s="104">
+        <v>10</v>
+      </c>
+      <c r="G13" s="102">
+        <v>313.57</v>
+      </c>
+      <c r="H13" s="102">
+        <f>708.66+95.83</f>
+        <v>804.49</v>
+      </c>
+      <c r="I13" s="102">
+        <v>575.16</v>
+      </c>
+      <c r="J13" s="12">
+        <v>366.18</v>
+      </c>
+      <c r="K13" s="12">
+        <f t="shared" si="0"/>
+        <v>2059.3999999999996</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="43.5">
+      <c r="A14" s="99">
+        <v>3</v>
+      </c>
+      <c r="B14" s="100">
+        <v>70</v>
+      </c>
+      <c r="C14" s="104" t="s">
+        <v>206</v>
+      </c>
+      <c r="D14" s="104">
+        <f>2.3+3.7</f>
+        <v>6</v>
+      </c>
+      <c r="E14" s="104" t="s">
+        <v>207</v>
+      </c>
+      <c r="F14" s="104">
+        <v>8</v>
+      </c>
+      <c r="G14" s="102">
+        <f>366.06*2</f>
+        <v>732.12</v>
+      </c>
+      <c r="H14" s="102">
+        <f>598.35+594.02</f>
+        <v>1192.3699999999999</v>
+      </c>
+      <c r="I14" s="102">
+        <f>(689.34+58.58)*2</f>
+        <v>1495.8400000000001</v>
+      </c>
+      <c r="J14" s="12">
+        <f>409.4+407.1</f>
+        <v>816.5</v>
+      </c>
+      <c r="K14" s="12">
+        <f t="shared" si="0"/>
+        <v>4236.83</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" ht="43.5">
+      <c r="A15" s="99">
+        <v>3</v>
+      </c>
+      <c r="B15" s="100">
+        <v>70</v>
+      </c>
+      <c r="C15" s="104" t="s">
+        <v>209</v>
+      </c>
+      <c r="D15" s="104">
+        <f>4.8+3.3</f>
+        <v>8.1</v>
+      </c>
+      <c r="E15" s="104" t="s">
+        <v>207</v>
+      </c>
+      <c r="F15" s="104">
+        <v>8</v>
+      </c>
+      <c r="G15" s="102">
+        <f>366.06*2</f>
+        <v>732.12</v>
+      </c>
+      <c r="H15" s="102">
+        <f>579.26+590.49</f>
+        <v>1169.75</v>
+      </c>
+      <c r="I15" s="102">
+        <f>(689.34+58.58)*2</f>
+        <v>1495.8400000000001</v>
+      </c>
+      <c r="J15" s="12">
+        <f>386.4+388.7</f>
+        <v>775.09999999999991</v>
+      </c>
+      <c r="K15" s="12">
+        <f t="shared" si="0"/>
+        <v>4172.8099999999995</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" ht="43.5">
+      <c r="A16" s="99">
+        <v>3</v>
+      </c>
+      <c r="B16" s="100">
+        <v>70</v>
+      </c>
+      <c r="C16" s="104" t="s">
+        <v>211</v>
+      </c>
+      <c r="D16" s="104">
+        <f>4.3+3.8</f>
+        <v>8.1</v>
+      </c>
+      <c r="E16" s="104" t="s">
+        <v>207</v>
+      </c>
+      <c r="F16" s="104">
+        <v>8</v>
+      </c>
+      <c r="G16" s="102">
+        <f>366.06+377.28</f>
+        <v>743.33999999999992</v>
+      </c>
+      <c r="H16" s="102">
+        <f>587.63+650.24</f>
+        <v>1237.8699999999999</v>
+      </c>
+      <c r="I16" s="102">
+        <f>493.14+51.28+471.71+60.82</f>
+        <v>1076.9499999999998</v>
+      </c>
+      <c r="J16" s="12">
+        <f>410.55+426.65</f>
+        <v>837.2</v>
+      </c>
+      <c r="K16" s="12">
+        <f t="shared" si="0"/>
+        <v>3895.3599999999997</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17" s="99">
+        <v>3</v>
+      </c>
+      <c r="B17" s="100">
+        <v>51.7</v>
+      </c>
+      <c r="C17" s="104" t="s">
+        <v>213</v>
+      </c>
+      <c r="D17" s="104">
+        <v>3</v>
+      </c>
+      <c r="E17" s="104" t="s">
+        <v>214</v>
+      </c>
+      <c r="F17" s="104">
+        <v>14</v>
+      </c>
+      <c r="G17" s="102">
+        <v>1082.9100000000001</v>
+      </c>
+      <c r="H17" s="102">
+        <v>2300.6</v>
+      </c>
+      <c r="I17" s="102">
+        <v>0</v>
+      </c>
+      <c r="J17" s="12">
+        <v>0</v>
+      </c>
+      <c r="K17" s="12">
+        <f t="shared" si="0"/>
+        <v>3383.51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" s="99">
+        <v>6</v>
+      </c>
+      <c r="B18" s="100">
+        <v>25</v>
+      </c>
+      <c r="C18" s="104" t="s">
+        <v>215</v>
+      </c>
+      <c r="D18" s="104">
+        <v>1</v>
+      </c>
+      <c r="E18" s="104" t="s">
+        <v>188</v>
+      </c>
+      <c r="F18" s="104">
+        <v>6</v>
+      </c>
+      <c r="G18" s="102">
+        <v>4512</v>
+      </c>
+      <c r="H18" s="102">
+        <v>4225.2</v>
+      </c>
+      <c r="I18" s="102">
+        <v>0</v>
+      </c>
+      <c r="J18" s="12">
+        <v>0</v>
+      </c>
+      <c r="K18" s="12">
+        <f t="shared" si="0"/>
+        <v>8737.2000000000007</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="29">
+      <c r="A19" s="105">
+        <v>3</v>
+      </c>
+      <c r="B19" s="105">
+        <v>44</v>
+      </c>
+      <c r="C19" s="106" t="s">
+        <v>217</v>
+      </c>
+      <c r="D19" s="106">
+        <f>5+5</f>
+        <v>10</v>
+      </c>
+      <c r="E19" s="106" t="s">
+        <v>218</v>
+      </c>
+      <c r="F19" s="106">
+        <v>12</v>
+      </c>
+      <c r="G19" s="107">
+        <f>308+226</f>
+        <v>534</v>
+      </c>
+      <c r="H19" s="107">
+        <f>478+489</f>
+        <v>967</v>
+      </c>
+      <c r="I19" s="107">
+        <v>0</v>
+      </c>
+      <c r="J19" s="108">
+        <v>0</v>
+      </c>
+      <c r="K19" s="108">
+        <f t="shared" si="0"/>
+        <v>1501</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" s="99">
+        <v>3</v>
+      </c>
+      <c r="B20" s="99">
+        <v>28.1</v>
+      </c>
+      <c r="C20" s="104" t="s">
+        <v>220</v>
+      </c>
+      <c r="D20" s="104">
+        <v>26</v>
+      </c>
+      <c r="E20" s="104" t="s">
+        <v>221</v>
+      </c>
+      <c r="F20" s="104">
+        <v>12.75</v>
+      </c>
+      <c r="G20" s="102">
+        <v>134.69999999999999</v>
+      </c>
+      <c r="H20" s="102">
+        <v>323</v>
+      </c>
+      <c r="I20" s="102">
+        <v>337.5</v>
+      </c>
+      <c r="J20" s="12">
+        <v>91.7</v>
+      </c>
+      <c r="K20" s="12">
+        <f t="shared" si="0"/>
+        <v>886.90000000000009</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21" s="99">
+        <v>3</v>
+      </c>
+      <c r="B21" s="99">
+        <v>91</v>
+      </c>
+      <c r="C21" s="104" t="s">
+        <v>223</v>
+      </c>
+      <c r="D21" s="104">
+        <v>17</v>
+      </c>
+      <c r="E21" s="104" t="s">
+        <v>207</v>
+      </c>
+      <c r="F21" s="104">
+        <v>8</v>
+      </c>
+      <c r="G21" s="102">
+        <f>414+204</f>
+        <v>618</v>
+      </c>
+      <c r="H21" s="102">
+        <f>1021+1001</f>
+        <v>2022</v>
+      </c>
+      <c r="I21" s="102">
+        <f>617+600</f>
+        <v>1217</v>
+      </c>
+      <c r="J21" s="12">
+        <f>493+91</f>
+        <v>584</v>
+      </c>
+      <c r="K21" s="12">
+        <f t="shared" si="0"/>
+        <v>4441</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="29">
+      <c r="A22" s="99">
+        <v>1</v>
+      </c>
+      <c r="B22" s="99">
+        <v>80</v>
+      </c>
+      <c r="C22" s="104" t="s">
+        <v>225</v>
+      </c>
+      <c r="D22" s="104">
+        <f>1+2.8</f>
+        <v>3.8</v>
+      </c>
+      <c r="E22" s="104" t="s">
+        <v>226</v>
+      </c>
+      <c r="F22" s="104">
+        <v>12</v>
+      </c>
+      <c r="G22" s="102">
+        <v>650.46</v>
+      </c>
+      <c r="H22" s="102">
+        <v>1451.5</v>
+      </c>
+      <c r="I22" s="102">
+        <v>1056</v>
+      </c>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12">
+        <f t="shared" si="0"/>
+        <v>3157.96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
+      <c r="A23" s="99">
+        <v>3</v>
+      </c>
+      <c r="B23" s="99">
+        <v>95.5</v>
+      </c>
+      <c r="C23" s="104" t="s">
+        <v>228</v>
+      </c>
+      <c r="D23" s="104">
+        <v>12.3</v>
+      </c>
+      <c r="E23" s="104" t="s">
+        <v>226</v>
+      </c>
+      <c r="F23" s="104">
+        <v>12</v>
+      </c>
+      <c r="G23" s="102">
+        <v>425</v>
+      </c>
+      <c r="H23" s="102">
+        <v>890</v>
+      </c>
+      <c r="I23" s="102">
+        <v>0</v>
+      </c>
+      <c r="J23" s="12">
+        <v>0</v>
+      </c>
+      <c r="K23" s="12">
+        <f t="shared" si="0"/>
+        <v>1315</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
+      <c r="A24" s="99">
+        <v>3</v>
+      </c>
+      <c r="B24" s="99">
+        <v>80</v>
+      </c>
+      <c r="C24" s="104" t="s">
+        <v>230</v>
+      </c>
+      <c r="D24" s="104">
+        <v>54</v>
+      </c>
+      <c r="E24" s="104" t="s">
+        <v>214</v>
+      </c>
+      <c r="F24" s="104">
+        <v>14</v>
+      </c>
+      <c r="G24" s="102">
+        <f>603*2</f>
+        <v>1206</v>
+      </c>
+      <c r="H24" s="102">
+        <f>972*2</f>
+        <v>1944</v>
+      </c>
+      <c r="I24" s="102">
+        <f>689+639</f>
+        <v>1328</v>
+      </c>
+      <c r="J24" s="12">
+        <v>0</v>
+      </c>
+      <c r="K24" s="12">
+        <f t="shared" si="0"/>
+        <v>4478</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
+      <c r="A25" s="99">
+        <v>3</v>
+      </c>
+      <c r="B25" s="102"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="102">
+        <v>450</v>
+      </c>
+      <c r="H25" s="102">
+        <v>860</v>
+      </c>
+      <c r="I25" s="102"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12">
+        <f t="shared" si="0"/>
+        <v>1310</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
+      <c r="A26" s="99">
+        <v>3</v>
+      </c>
+      <c r="B26" s="102"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="102">
+        <v>450</v>
+      </c>
+      <c r="H26" s="102">
+        <v>860</v>
+      </c>
+      <c r="I26" s="102"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="12">
+        <f t="shared" si="0"/>
+        <v>1310</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
+      <c r="A27" s="99">
+        <v>4</v>
+      </c>
+      <c r="B27" s="99">
+        <v>22.92</v>
+      </c>
+      <c r="C27" s="109">
+        <v>9</v>
+      </c>
+      <c r="D27" s="55"/>
+      <c r="E27" s="109" t="s">
+        <v>199</v>
+      </c>
+      <c r="F27" s="109">
+        <v>10</v>
+      </c>
+      <c r="G27" s="102">
+        <v>640.79</v>
+      </c>
+      <c r="H27" s="102">
+        <v>585.49</v>
+      </c>
+      <c r="I27" s="102">
+        <v>459.81</v>
+      </c>
+      <c r="J27" s="55"/>
+      <c r="K27" s="55">
+        <f t="shared" si="0"/>
+        <v>1686.09</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
+      <c r="A28" s="99">
+        <v>4</v>
+      </c>
+      <c r="B28" s="99">
+        <v>41</v>
+      </c>
+      <c r="C28" s="104">
+        <v>28</v>
+      </c>
+      <c r="D28" s="12"/>
+      <c r="E28" s="104">
+        <v>18</v>
+      </c>
+      <c r="F28" s="104">
+        <v>18</v>
+      </c>
+      <c r="G28" s="102">
+        <v>900.61</v>
+      </c>
+      <c r="H28" s="102">
+        <f>684.55+72</f>
+        <v>756.55</v>
+      </c>
+      <c r="I28" s="102">
+        <v>79</v>
+      </c>
+      <c r="J28" s="12">
+        <v>731.22</v>
+      </c>
+      <c r="K28" s="12">
+        <f>SUM(G28:J28)</f>
+        <v>2467.38</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11">
+      <c r="A29" s="99">
+        <v>6</v>
+      </c>
+      <c r="B29" s="99">
+        <v>71.900000000000006</v>
+      </c>
+      <c r="C29" s="104"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="104"/>
+      <c r="F29" s="104"/>
+      <c r="G29" s="102">
+        <v>5957</v>
+      </c>
+      <c r="H29" s="102">
+        <v>5383</v>
+      </c>
+      <c r="I29" s="102"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="12">
+        <f>SUM(G29:J29)</f>
+        <v>11340</v>
+      </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="S1" r:id="rId1" xr:uid="{FFCE48F2-C7C4-40DB-8D55-3EF2C21D7317}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>